<commit_message>
Trained 10 more models, but they may not be worth keeping...
</commit_message>
<xml_diff>
--- a/data/c_vs_random1_checkers.xlsx
+++ b/data/c_vs_random1_checkers.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -775,6 +775,116 @@
         <v>23.977</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="1" t="n">
+        <v>106</v>
+      </c>
+      <c r="B32" t="n">
+        <v>43</v>
+      </c>
+      <c r="C32" t="n">
+        <v>23.508</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n">
+        <v>108</v>
+      </c>
+      <c r="B33" t="n">
+        <v>46.8</v>
+      </c>
+      <c r="C33" t="n">
+        <v>23.987</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n">
+        <v>110</v>
+      </c>
+      <c r="B34" t="n">
+        <v>45</v>
+      </c>
+      <c r="C34" t="n">
+        <v>23.465</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n">
+        <v>112</v>
+      </c>
+      <c r="B35" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="C35" t="n">
+        <v>24.093</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n">
+        <v>114</v>
+      </c>
+      <c r="B36" t="n">
+        <v>45.8</v>
+      </c>
+      <c r="C36" t="n">
+        <v>23.832</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n">
+        <v>116</v>
+      </c>
+      <c r="B37" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="C37" t="n">
+        <v>24.338</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n">
+        <v>118</v>
+      </c>
+      <c r="B38" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="C38" t="n">
+        <v>24.029</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="n">
+        <v>120</v>
+      </c>
+      <c r="B39" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="C39" t="n">
+        <v>23.724</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="n">
+        <v>122</v>
+      </c>
+      <c r="B40" t="n">
+        <v>44.3</v>
+      </c>
+      <c r="C40" t="n">
+        <v>23.862</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n">
+        <v>124</v>
+      </c>
+      <c r="B41" t="n">
+        <v>44.3</v>
+      </c>
+      <c r="C41" t="n">
+        <v>24.411</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>